<commit_message>
growth factor updates for AEO 2026
</commit_message>
<xml_diff>
--- a/growth_factors/growth_factors.xlsx
+++ b/growth_factors/growth_factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ewilson/Documents/code/buildstock-weatherreg/growth_factors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F562DAD-2C13-0143-BB92-F240993C3B45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C385E09C-9204-0048-9668-BDA0F338D9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-2900" windowWidth="51200" windowHeight="28300" activeTab="4" xr2:uid="{5073E79D-3BF6-0D4F-A91F-B44D405A9A3E}"/>
+    <workbookView xWindow="5300" yWindow="12340" windowWidth="14400" windowHeight="9660" activeTab="4" xr2:uid="{5073E79D-3BF6-0D4F-A91F-B44D405A9A3E}"/>
   </bookViews>
   <sheets>
     <sheet name="baseline" sheetId="1" r:id="rId1"/>
@@ -7545,7 +7545,7 @@
         <v>3.1368719999999999</v>
       </c>
       <c r="D5">
-        <f t="shared" ref="D4:D28" si="14">C5+D4</f>
+        <f t="shared" ref="D5:D28" si="14">C5+D4</f>
         <v>3.1368719999999999</v>
       </c>
       <c r="E5">
@@ -7581,11 +7581,11 @@
         <v>133.665718</v>
       </c>
       <c r="N5">
-        <f t="shared" ref="N4:Q28" si="15">J5-R5</f>
+        <f t="shared" ref="N5:Q28" si="15">J5-R5</f>
         <v>0</v>
       </c>
       <c r="O5">
-        <f t="shared" ref="O2:Q17" si="16">K5-S5</f>
+        <f t="shared" ref="O5:Q17" si="16">K5-S5</f>
         <v>0</v>
       </c>
       <c r="P5">
@@ -7705,7 +7705,7 @@
         <v>3.8291843999999995</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G2:G28" si="17">B6-D6</f>
+        <f t="shared" ref="G6:G28" si="17">B6-D6</f>
         <v>102.812865</v>
       </c>
       <c r="H6">
@@ -7745,7 +7745,7 @@
         <v>2.4150058231152514</v>
       </c>
       <c r="R6">
-        <f t="shared" ref="R4:U19" si="18">R5*(1-$V5)</f>
+        <f t="shared" ref="R6:U19" si="18">R5*(1-$V5)</f>
         <v>90.992935300413194</v>
       </c>
       <c r="S6">
@@ -11763,7 +11763,7 @@
         <v>133.665718</v>
       </c>
       <c r="N5">
-        <f t="shared" ref="N5:Q29" si="15">J5-R5</f>
+        <f t="shared" ref="N5:Q28" si="15">J5-R5</f>
         <v>0</v>
       </c>
       <c r="O5">
@@ -11887,7 +11887,7 @@
         <v>3.8291843999999995</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G32" si="16">B6-D6</f>
+        <f t="shared" ref="G6:G28" si="16">B6-D6</f>
         <v>102.812865</v>
       </c>
       <c r="H6">
@@ -15933,7 +15933,7 @@
         <v>133.665718</v>
       </c>
       <c r="N5">
-        <f t="shared" ref="N5:Q29" si="15">J5-R5</f>
+        <f t="shared" ref="N5:Q28" si="15">J5-R5</f>
         <v>0</v>
       </c>
       <c r="O5">
@@ -15986,7 +15986,7 @@
       </c>
       <c r="AA5">
         <f>MIN(AA4+(AA$28/20),AA$28)</f>
-        <v>0.04</v>
+        <v>2.7500000000000004E-2</v>
       </c>
       <c r="AB5">
         <v>1</v>
@@ -16004,7 +16004,7 @@
       </c>
       <c r="AF5">
         <f t="shared" si="7"/>
-        <v>2.5051753920000004</v>
+        <v>1.7223080820000003</v>
       </c>
       <c r="AG5">
         <f>$AC5*F5</f>
@@ -16024,7 +16024,7 @@
       </c>
       <c r="AK5">
         <f t="shared" si="11"/>
-        <v>60.124209408000006</v>
+        <v>60.907076718000006</v>
       </c>
       <c r="AL5">
         <f t="shared" si="12"/>
@@ -16060,7 +16060,7 @@
         <v>3.8291843999999995</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G32" si="16">B6-D6</f>
+        <f t="shared" ref="G6:G28" si="16">B6-D6</f>
         <v>102.812865</v>
       </c>
       <c r="H6">
@@ -16137,7 +16137,7 @@
       </c>
       <c r="AA6">
         <f t="shared" ref="AA6:AA27" si="19">MIN(AA5+(AA$28/20),AA$28)</f>
-        <v>0.08</v>
+        <v>5.5000000000000007E-2</v>
       </c>
       <c r="AB6">
         <v>1</v>
@@ -16155,7 +16155,7 @@
       </c>
       <c r="AF6">
         <f t="shared" si="7"/>
-        <v>4.9350175200000006</v>
+        <v>3.3928245450000003</v>
       </c>
       <c r="AG6">
         <f t="shared" ref="AG6:AG28" si="20">$AC6*F6</f>
@@ -16175,7 +16175,7 @@
       </c>
       <c r="AK6">
         <f t="shared" si="11"/>
-        <v>56.752701479999999</v>
+        <v>58.294894454999998</v>
       </c>
       <c r="AL6">
         <f t="shared" si="12"/>
@@ -16288,7 +16288,7 @@
       </c>
       <c r="AA7">
         <f t="shared" si="19"/>
-        <v>0.12</v>
+        <v>8.2500000000000018E-2</v>
       </c>
       <c r="AB7">
         <v>1</v>
@@ -16306,7 +16306,7 @@
       </c>
       <c r="AF7">
         <f t="shared" si="7"/>
-        <v>7.288179551999999</v>
+        <v>5.0106234420000009</v>
       </c>
       <c r="AG7">
         <f t="shared" si="20"/>
@@ -16326,7 +16326,7 @@
       </c>
       <c r="AK7">
         <f t="shared" si="11"/>
-        <v>53.446650047999995</v>
+        <v>55.724206157999994</v>
       </c>
       <c r="AL7">
         <f t="shared" si="12"/>
@@ -16439,7 +16439,7 @@
       </c>
       <c r="AA8">
         <f t="shared" si="19"/>
-        <v>0.16</v>
+        <v>0.11000000000000001</v>
       </c>
       <c r="AB8">
         <v>1</v>
@@ -16457,7 +16457,7 @@
       </c>
       <c r="AF8">
         <f t="shared" si="7"/>
-        <v>9.5631964800000002</v>
+        <v>6.5746975800000005</v>
       </c>
       <c r="AG8">
         <f t="shared" si="20"/>
@@ -16477,7 +16477,7 @@
       </c>
       <c r="AK8">
         <f t="shared" si="11"/>
-        <v>50.206781519999993</v>
+        <v>53.195280419999996</v>
       </c>
       <c r="AL8">
         <f t="shared" si="12"/>
@@ -16590,7 +16590,7 @@
       </c>
       <c r="AA9">
         <f t="shared" si="19"/>
-        <v>0.2</v>
+        <v>0.13750000000000001</v>
       </c>
       <c r="AB9">
         <v>1</v>
@@ -16608,7 +16608,7 @@
       </c>
       <c r="AF9">
         <f t="shared" si="7"/>
-        <v>11.758565040000001</v>
+        <v>8.0840134650000017</v>
       </c>
       <c r="AG9">
         <f t="shared" si="20"/>
@@ -16628,7 +16628,7 @@
       </c>
       <c r="AK9">
         <f t="shared" si="11"/>
-        <v>47.034260160000002</v>
+        <v>50.708811734999998</v>
       </c>
       <c r="AL9">
         <f t="shared" si="12"/>
@@ -16741,7 +16741,7 @@
       </c>
       <c r="AA10">
         <f t="shared" si="19"/>
-        <v>0.24000000000000002</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="AB10">
         <v>1</v>
@@ -16759,7 +16759,7 @@
       </c>
       <c r="AF10">
         <f t="shared" si="7"/>
-        <v>13.872756528</v>
+        <v>9.5375201129999994</v>
       </c>
       <c r="AG10">
         <f t="shared" si="20"/>
@@ -16779,7 +16779,7 @@
       </c>
       <c r="AK10">
         <f t="shared" si="11"/>
-        <v>43.930395671999989</v>
+        <v>48.265632086999993</v>
       </c>
       <c r="AL10">
         <f t="shared" si="12"/>
@@ -16892,7 +16892,7 @@
       </c>
       <c r="AA11">
         <f t="shared" si="19"/>
-        <v>0.28000000000000003</v>
+        <v>0.1925</v>
       </c>
       <c r="AB11">
         <v>1</v>
@@ -16910,7 +16910,7 @@
       </c>
       <c r="AF11">
         <f t="shared" si="7"/>
-        <v>15.904191072</v>
+        <v>10.934131361999999</v>
       </c>
       <c r="AG11">
         <f t="shared" si="20"/>
@@ -16930,7 +16930,7 @@
       </c>
       <c r="AK11">
         <f t="shared" si="11"/>
-        <v>40.896491327999996</v>
+        <v>45.866551037999997</v>
       </c>
       <c r="AL11">
         <f t="shared" si="12"/>
@@ -17043,7 +17043,7 @@
       </c>
       <c r="AA12">
         <f t="shared" si="19"/>
-        <v>0.32</v>
+        <v>0.22</v>
       </c>
       <c r="AB12">
         <v>1</v>
@@ -17061,7 +17061,7 @@
       </c>
       <c r="AF12">
         <f t="shared" si="7"/>
-        <v>17.851228799999998</v>
+        <v>12.272719799999999</v>
       </c>
       <c r="AG12">
         <f t="shared" si="20"/>
@@ -17081,7 +17081,7 @@
       </c>
       <c r="AK12">
         <f t="shared" si="11"/>
-        <v>37.933861199999996</v>
+        <v>43.512370199999999</v>
       </c>
       <c r="AL12">
         <f t="shared" si="12"/>
@@ -17194,7 +17194,7 @@
       </c>
       <c r="AA13">
         <f t="shared" si="19"/>
-        <v>0.36</v>
+        <v>0.2475</v>
       </c>
       <c r="AB13">
         <v>1</v>
@@ -17212,7 +17212,7 @@
       </c>
       <c r="AF13">
         <f t="shared" si="7"/>
-        <v>19.712201687999997</v>
+        <v>13.552138660499999</v>
       </c>
       <c r="AG13">
         <f t="shared" si="20"/>
@@ -17232,7 +17232,7 @@
       </c>
       <c r="AK13">
         <f t="shared" si="11"/>
-        <v>35.043914111999996</v>
+        <v>41.203977139499997</v>
       </c>
       <c r="AL13">
         <f t="shared" si="12"/>
@@ -17345,7 +17345,7 @@
       </c>
       <c r="AA14">
         <f t="shared" si="19"/>
-        <v>0.39999999999999997</v>
+        <v>0.27500000000000002</v>
       </c>
       <c r="AB14">
         <v>1</v>
@@ -17363,7 +17363,7 @@
       </c>
       <c r="AF14">
         <f t="shared" si="7"/>
-        <v>21.485428559999995</v>
+        <v>14.771232134999998</v>
       </c>
       <c r="AG14">
         <f t="shared" si="20"/>
@@ -17383,7 +17383,7 @@
       </c>
       <c r="AK14">
         <f t="shared" si="11"/>
-        <v>32.228142839999997</v>
+        <v>38.942339264999994</v>
       </c>
       <c r="AL14">
         <f t="shared" si="12"/>
@@ -17496,7 +17496,7 @@
       </c>
       <c r="AA15">
         <f t="shared" si="19"/>
-        <v>0.43999999999999995</v>
+        <v>0.30250000000000005</v>
       </c>
       <c r="AB15">
         <v>1</v>
@@ -17514,7 +17514,7 @@
       </c>
       <c r="AF15">
         <f t="shared" si="7"/>
-        <v>23.169257231999996</v>
+        <v>15.928864347000003</v>
       </c>
       <c r="AG15">
         <f t="shared" si="20"/>
@@ -17534,7 +17534,7 @@
       </c>
       <c r="AK15">
         <f t="shared" si="11"/>
-        <v>29.488145568000004</v>
+        <v>36.728538452999999</v>
       </c>
       <c r="AL15">
         <f t="shared" si="12"/>
@@ -17647,7 +17647,7 @@
       </c>
       <c r="AA16">
         <f t="shared" si="19"/>
-        <v>0.47999999999999993</v>
+        <v>0.33000000000000007</v>
       </c>
       <c r="AB16">
         <v>1</v>
@@ -17665,7 +17665,7 @@
       </c>
       <c r="AF16">
         <f t="shared" si="7"/>
-        <v>24.762070368</v>
+        <v>17.023923378000006</v>
       </c>
       <c r="AG16">
         <f t="shared" si="20"/>
@@ -17685,7 +17685,7 @@
       </c>
       <c r="AK16">
         <f t="shared" si="11"/>
-        <v>26.825576232000007</v>
+        <v>34.563723222</v>
       </c>
       <c r="AL16">
         <f t="shared" si="12"/>
@@ -17798,7 +17798,7 @@
       </c>
       <c r="AA17">
         <f t="shared" si="19"/>
-        <v>0.51999999999999991</v>
+        <v>0.3575000000000001</v>
       </c>
       <c r="AB17">
         <v>1</v>
@@ -17816,7 +17816,7 @@
       </c>
       <c r="AF17">
         <f t="shared" si="7"/>
-        <v>26.262281447999996</v>
+        <v>18.055318495500003</v>
       </c>
       <c r="AG17">
         <f t="shared" si="20"/>
@@ -17836,7 +17836,7 @@
       </c>
       <c r="AK17">
         <f t="shared" si="11"/>
-        <v>24.242105952000003</v>
+        <v>32.449068904499995</v>
       </c>
       <c r="AL17">
         <f t="shared" si="12"/>
@@ -17949,7 +17949,7 @@
       </c>
       <c r="AA18">
         <f t="shared" si="19"/>
-        <v>0.55999999999999994</v>
+        <v>0.38500000000000012</v>
       </c>
       <c r="AB18">
         <v>1</v>
@@ -17967,7 +17967,7 @@
       </c>
       <c r="AF18">
         <f t="shared" si="7"/>
-        <v>27.668318160000005</v>
+        <v>19.021968735000012</v>
       </c>
       <c r="AG18">
         <f t="shared" si="20"/>
@@ -17987,7 +17987,7 @@
       </c>
       <c r="AK18">
         <f t="shared" si="11"/>
-        <v>21.739392840000008</v>
+        <v>30.385742265000001</v>
       </c>
       <c r="AL18">
         <f t="shared" si="12"/>
@@ -18100,7 +18100,7 @@
       </c>
       <c r="AA19">
         <f t="shared" si="19"/>
-        <v>0.6</v>
+        <v>0.41250000000000014</v>
       </c>
       <c r="AB19">
         <v>1</v>
@@ -18118,7 +18118,7 @@
       </c>
       <c r="AF19">
         <f t="shared" si="7"/>
-        <v>28.978634519999996</v>
+        <v>19.922811232500006</v>
       </c>
       <c r="AG19">
         <f t="shared" si="20"/>
@@ -18138,7 +18138,7 @@
       </c>
       <c r="AK19">
         <f t="shared" si="11"/>
-        <v>19.319089680000001</v>
+        <v>28.374912967499991</v>
       </c>
       <c r="AL19">
         <f t="shared" si="12"/>
@@ -18251,7 +18251,7 @@
       </c>
       <c r="AA20">
         <f t="shared" si="19"/>
-        <v>0.64</v>
+        <v>0.44000000000000017</v>
       </c>
       <c r="AB20">
         <v>1</v>
@@ -18269,7 +18269,7 @@
       </c>
       <c r="AF20">
         <f t="shared" si="7"/>
-        <v>30.191685120000002</v>
+        <v>20.75678352000001</v>
       </c>
       <c r="AG20">
         <f t="shared" si="20"/>
@@ -18289,7 +18289,7 @@
       </c>
       <c r="AK20">
         <f t="shared" si="11"/>
-        <v>16.982822880000001</v>
+        <v>26.417724479999993</v>
       </c>
       <c r="AL20">
         <f t="shared" si="12"/>
@@ -18402,7 +18402,7 @@
       </c>
       <c r="AA21">
         <f t="shared" si="19"/>
-        <v>0.68</v>
+        <v>0.46750000000000019</v>
       </c>
       <c r="AB21">
         <v>1</v>
@@ -18420,7 +18420,7 @@
       </c>
       <c r="AF21">
         <f t="shared" si="7"/>
-        <v>31.305955872000002</v>
+        <v>21.522844662000008</v>
       </c>
       <c r="AG21">
         <f t="shared" si="20"/>
@@ -18440,7 +18440,7 @@
       </c>
       <c r="AK21">
         <f t="shared" si="11"/>
-        <v>14.732214527999997</v>
+        <v>24.515325737999991</v>
       </c>
       <c r="AL21">
         <f t="shared" si="12"/>
@@ -18553,7 +18553,7 @@
       </c>
       <c r="AA22">
         <f t="shared" si="19"/>
-        <v>0.72000000000000008</v>
+        <v>0.49500000000000022</v>
       </c>
       <c r="AB22">
         <v>1</v>
@@ -18571,7 +18571,7 @@
       </c>
       <c r="AF22">
         <f t="shared" si="7"/>
-        <v>32.319902448000001</v>
+        <v>22.21993293300001</v>
       </c>
       <c r="AG22">
         <f t="shared" si="20"/>
@@ -18591,7 +18591,7 @@
       </c>
       <c r="AK22">
         <f t="shared" si="11"/>
-        <v>12.568850951999998</v>
+        <v>22.668820466999989</v>
       </c>
       <c r="AL22">
         <f t="shared" si="12"/>
@@ -18704,7 +18704,7 @@
       </c>
       <c r="AA23">
         <f t="shared" si="19"/>
-        <v>0.76000000000000012</v>
+        <v>0.52250000000000019</v>
       </c>
       <c r="AB23">
         <v>1</v>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="AF23">
         <f t="shared" si="7"/>
-        <v>33.232009584000011</v>
+        <v>22.847006589000014</v>
       </c>
       <c r="AG23">
         <f t="shared" si="20"/>
@@ -18742,7 +18742,7 @@
       </c>
       <c r="AK23">
         <f t="shared" si="11"/>
-        <v>10.494318815999996</v>
+        <v>20.879321810999993</v>
       </c>
       <c r="AL23">
         <f t="shared" si="12"/>
@@ -18855,7 +18855,7 @@
       </c>
       <c r="AA24">
         <f t="shared" si="19"/>
-        <v>0.8</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AB24">
         <v>1</v>
@@ -18873,7 +18873,7 @@
       </c>
       <c r="AF24">
         <f t="shared" si="7"/>
-        <v>34.04072544000001</v>
+        <v>23.402998740000008</v>
       </c>
       <c r="AG24">
         <f t="shared" si="20"/>
@@ -18893,7 +18893,7 @@
       </c>
       <c r="AK24">
         <f t="shared" si="11"/>
-        <v>8.5101813600000042</v>
+        <v>19.147908060000006</v>
       </c>
       <c r="AL24">
         <f t="shared" si="12"/>
@@ -19006,7 +19006,7 @@
       </c>
       <c r="AA25">
         <f t="shared" si="19"/>
-        <v>0.8</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AB25">
         <v>1</v>
@@ -19024,7 +19024,7 @@
       </c>
       <c r="AF25">
         <f t="shared" si="7"/>
-        <v>33.090022560000016</v>
+        <v>22.749390510000008</v>
       </c>
       <c r="AG25">
         <f t="shared" si="20"/>
@@ -19044,7 +19044,7 @@
       </c>
       <c r="AK25">
         <f t="shared" si="11"/>
-        <v>8.2725056399999986</v>
+        <v>18.613137690000006</v>
       </c>
       <c r="AL25">
         <f t="shared" si="12"/>
@@ -19054,8 +19054,7 @@
         <v>0.4</v>
       </c>
       <c r="AN25">
-        <f>MIN(AN24+(1/20),AN$28)</f>
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:40" x14ac:dyDescent="0.2">
@@ -19158,7 +19157,7 @@
       </c>
       <c r="AA26">
         <f t="shared" si="19"/>
-        <v>0.8</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AB26">
         <v>1</v>
@@ -19176,7 +19175,7 @@
       </c>
       <c r="AF26">
         <f t="shared" si="7"/>
-        <v>32.12893536</v>
+        <v>22.088643059999999</v>
       </c>
       <c r="AG26">
         <f t="shared" si="20"/>
@@ -19196,7 +19195,7 @@
       </c>
       <c r="AK26">
         <f t="shared" si="11"/>
-        <v>8.0322338399999964</v>
+        <v>18.072526139999997</v>
       </c>
       <c r="AL26">
         <f t="shared" si="12"/>
@@ -19206,8 +19205,7 @@
         <v>0.4</v>
       </c>
       <c r="AN26">
-        <f>MIN(AN25+(1/20),AN$28)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:40" x14ac:dyDescent="0.2">
@@ -19310,7 +19308,7 @@
       </c>
       <c r="AA27">
         <f t="shared" si="19"/>
-        <v>0.8</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AB27">
         <v>1</v>
@@ -19328,7 +19326,7 @@
       </c>
       <c r="AF27">
         <f t="shared" si="7"/>
-        <v>31.157457120000004</v>
+        <v>21.420751770000003</v>
       </c>
       <c r="AG27">
         <f t="shared" si="20"/>
@@ -19348,7 +19346,7 @@
       </c>
       <c r="AK27">
         <f t="shared" si="11"/>
-        <v>7.7893642800000009</v>
+        <v>17.526069630000002</v>
       </c>
       <c r="AL27">
         <f t="shared" si="12"/>
@@ -19358,8 +19356,7 @@
         <v>0.4</v>
       </c>
       <c r="AN27">
-        <f>MIN(AN26+(1/20),AN$28)</f>
-        <v>0.15000000000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:40" x14ac:dyDescent="0.2">
@@ -19460,8 +19457,7 @@
         <v>0.8</v>
       </c>
       <c r="AA28">
-        <f>0.8</f>
-        <v>0.8</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="AB28">
         <v>1</v>
@@ -19479,7 +19475,7 @@
       </c>
       <c r="AF28">
         <f t="shared" si="7"/>
-        <v>30.175544639999998</v>
+        <v>20.745686939999999</v>
       </c>
       <c r="AG28">
         <f t="shared" si="20"/>
@@ -19499,7 +19495,7 @@
       </c>
       <c r="AK28">
         <f t="shared" si="11"/>
-        <v>7.5438861599999996</v>
+        <v>16.973743859999999</v>
       </c>
       <c r="AL28">
         <f t="shared" si="12"/>
@@ -19509,7 +19505,7 @@
         <v>0.4</v>
       </c>
       <c r="AN28">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:40" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Fix growth factor res demolition columns for MF and MH
</commit_message>
<xml_diff>
--- a/growth_factors/growth_factors.xlsx
+++ b/growth_factors/growth_factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ewilson/Documents/code/buildstock-weatherreg/growth_factors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C385E09C-9204-0048-9668-BDA0F338D9DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09D74782-67D5-0C43-885A-A314124EAC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5300" yWindow="12340" windowWidth="14400" windowHeight="9660" activeTab="4" xr2:uid="{5073E79D-3BF6-0D4F-A91F-B44D405A9A3E}"/>
+    <workbookView xWindow="8400" yWindow="4140" windowWidth="14400" windowHeight="9660" firstSheet="4" activeTab="4" xr2:uid="{5073E79D-3BF6-0D4F-A91F-B44D405A9A3E}"/>
   </bookViews>
   <sheets>
     <sheet name="baseline" sheetId="1" r:id="rId1"/>
@@ -15961,7 +15961,7 @@
         <v>6.7927460000000002</v>
       </c>
       <c r="U5">
-        <f>M5</f>
+        <f>SUM(R5:T5)</f>
         <v>133.665718</v>
       </c>
       <c r="V5">
@@ -16089,31 +16089,31 @@
       </c>
       <c r="O6">
         <f t="shared" si="15"/>
-        <v>0.71706116646421947</v>
+        <v>0.88283948056918149</v>
       </c>
       <c r="P6">
         <f t="shared" si="15"/>
-        <v>5.9415957064224756E-2</v>
+        <v>0.26286740047561352</v>
       </c>
       <c r="Q6">
         <f t="shared" si="15"/>
-        <v>2.4150058231152514</v>
+        <v>2.7842355806315879</v>
       </c>
       <c r="R6">
-        <f t="shared" ref="R6:U21" si="17">R5*(1-$V5)</f>
+        <f>R5*(1-V5)</f>
         <v>90.992935300413194</v>
       </c>
       <c r="S6">
-        <f t="shared" si="17"/>
-        <v>34.985150833535783</v>
+        <f t="shared" ref="S6:T6" si="17">S5*(1-W5)</f>
+        <v>34.819372519430821</v>
       </c>
       <c r="T6">
         <f t="shared" si="17"/>
-        <v>6.7448340429357749</v>
+        <v>6.5413825995243862</v>
       </c>
       <c r="U6">
-        <f t="shared" si="17"/>
-        <v>132.72292017688474</v>
+        <f t="shared" ref="U6:U28" si="18">SUM(R6:T6)</f>
+        <v>132.35369041936841</v>
       </c>
       <c r="V6">
         <f t="shared" si="13"/>
@@ -16132,11 +16132,11 @@
         <v>9.8045071674785524E-3</v>
       </c>
       <c r="Z6">
-        <f t="shared" ref="Z6:Z27" si="18">MIN(Z5+(Z$28/20),Z$28)</f>
+        <f t="shared" ref="Z6:Z27" si="19">MIN(Z5+(Z$28/20),Z$28)</f>
         <v>0.08</v>
       </c>
       <c r="AA6">
-        <f t="shared" ref="AA6:AA27" si="19">MIN(AA5+(AA$28/20),AA$28)</f>
+        <f t="shared" ref="AA6:AA27" si="20">MIN(AA5+(AA$28/20),AA$28)</f>
         <v>5.5000000000000007E-2</v>
       </c>
       <c r="AB6">
@@ -16147,18 +16147,18 @@
       </c>
       <c r="AD6">
         <f t="shared" si="5"/>
-        <v>10.617833614150779</v>
+        <v>10.588295233549472</v>
       </c>
       <c r="AE6">
         <f t="shared" si="6"/>
-        <v>2.4150058231152514</v>
+        <v>2.7842355806315879</v>
       </c>
       <c r="AF6">
         <f t="shared" si="7"/>
         <v>3.3928245450000003</v>
       </c>
       <c r="AG6">
-        <f t="shared" ref="AG6:AG28" si="20">$AC6*F6</f>
+        <f t="shared" ref="AG6:AG28" si="21">$AC6*F6</f>
         <v>3.8291843999999995</v>
       </c>
       <c r="AH6">
@@ -16167,7 +16167,7 @@
       </c>
       <c r="AI6">
         <f t="shared" si="9"/>
-        <v>122.10508656273396</v>
+        <v>121.76539518581893</v>
       </c>
       <c r="AJ6">
         <f t="shared" si="10"/>
@@ -16240,31 +16240,31 @@
       </c>
       <c r="O7">
         <f t="shared" si="15"/>
-        <v>1.4699614418576772</v>
+        <v>1.7983994630808695</v>
       </c>
       <c r="P7">
         <f t="shared" si="15"/>
-        <v>0.11665897191336949</v>
+        <v>0.51459817844117595</v>
       </c>
       <c r="Q7">
         <f t="shared" si="15"/>
-        <v>4.8611587157279814</v>
+        <v>5.5875359434789686</v>
       </c>
       <c r="R7">
-        <f t="shared" si="17"/>
+        <f t="shared" ref="R7:R28" si="22">R6*(1-V6)</f>
         <v>90.351125698043077</v>
       </c>
       <c r="S7">
-        <f t="shared" si="17"/>
-        <v>34.738386558142324</v>
+        <f t="shared" ref="S7:S28" si="23">S6*(1-W6)</f>
+        <v>34.409948536919131</v>
       </c>
       <c r="T7">
-        <f t="shared" si="17"/>
-        <v>6.6972600280866308</v>
+        <f t="shared" ref="T7:T28" si="24">T6*(1-X6)</f>
+        <v>6.2993208215588243</v>
       </c>
       <c r="U7">
-        <f t="shared" si="17"/>
-        <v>131.78677228427202</v>
+        <f t="shared" si="18"/>
+        <v>131.06039505652103</v>
       </c>
       <c r="V7">
         <f t="shared" si="13"/>
@@ -16283,11 +16283,11 @@
         <v>9.7936532884591015E-3</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.12</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>8.2500000000000018E-2</v>
       </c>
       <c r="AB7">
@@ -16298,18 +16298,18 @@
       </c>
       <c r="AD7">
         <f t="shared" si="5"/>
-        <v>15.814412674112642</v>
+        <v>15.727247406782523</v>
       </c>
       <c r="AE7">
         <f t="shared" si="6"/>
-        <v>4.8611587157279814</v>
+        <v>5.5875359434789686</v>
       </c>
       <c r="AF7">
         <f t="shared" si="7"/>
         <v>5.0106234420000009</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>5.7845813999999995</v>
       </c>
       <c r="AH7">
@@ -16318,7 +16318,7 @@
       </c>
       <c r="AI7">
         <f t="shared" si="9"/>
-        <v>115.97235961015937</v>
+        <v>115.33314764973851</v>
       </c>
       <c r="AJ7">
         <f t="shared" si="10"/>
@@ -16391,31 +16391,31 @@
       </c>
       <c r="O8">
         <f t="shared" si="15"/>
-        <v>2.2332051900228791</v>
+        <v>2.7212292290996558</v>
       </c>
       <c r="P8">
         <f t="shared" si="15"/>
-        <v>0.16896742818917332</v>
+        <v>0.75277253747268702</v>
       </c>
       <c r="Q8">
         <f t="shared" si="15"/>
-        <v>7.3018975824603558</v>
+        <v>8.3737267308206356</v>
       </c>
       <c r="R8">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>89.713843035751708</v>
       </c>
       <c r="S8">
-        <f t="shared" si="17"/>
-        <v>34.493362809977121</v>
+        <f t="shared" si="23"/>
+        <v>34.005338770900345</v>
       </c>
       <c r="T8">
-        <f t="shared" si="17"/>
-        <v>6.6500215718108269</v>
+        <f t="shared" si="24"/>
+        <v>6.0662164625273132</v>
       </c>
       <c r="U8">
-        <f t="shared" si="17"/>
-        <v>130.85722741753963</v>
+        <f t="shared" si="18"/>
+        <v>129.78539826917935</v>
       </c>
       <c r="V8">
         <f t="shared" si="13"/>
@@ -16434,11 +16434,11 @@
         <v>9.7824276944813507E-3</v>
       </c>
       <c r="Z8">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.16</v>
       </c>
       <c r="AA8">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.11000000000000001</v>
       </c>
       <c r="AB8">
@@ -16449,18 +16449,18 @@
       </c>
       <c r="AD8">
         <f t="shared" si="5"/>
-        <v>20.937156386806343</v>
+        <v>20.765663723068698</v>
       </c>
       <c r="AE8">
         <f t="shared" si="6"/>
-        <v>7.3018975824603558</v>
+        <v>8.3737267308206356</v>
       </c>
       <c r="AF8">
         <f t="shared" si="7"/>
         <v>6.5746975800000005</v>
       </c>
       <c r="AG8">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>7.7261723999999994</v>
       </c>
       <c r="AH8">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="AI8">
         <f t="shared" si="9"/>
-        <v>109.92007103073328</v>
+        <v>109.01973454611066</v>
       </c>
       <c r="AJ8">
         <f t="shared" si="10"/>
@@ -16542,31 +16542,31 @@
       </c>
       <c r="O9">
         <f t="shared" si="15"/>
-        <v>2.9974046875951998</v>
+        <v>3.641985386644194</v>
       </c>
       <c r="P9">
         <f t="shared" si="15"/>
-        <v>0.22225769272059726</v>
+        <v>0.98363594400253707</v>
       </c>
       <c r="Q9">
         <f t="shared" si="15"/>
-        <v>9.7377269970974965</v>
+        <v>11.143685947428423</v>
       </c>
       <c r="R9">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>89.081055383218313</v>
       </c>
       <c r="S9">
-        <f t="shared" si="17"/>
-        <v>34.250067312404802</v>
+        <f t="shared" si="23"/>
+        <v>33.605486613355808</v>
       </c>
       <c r="T9">
-        <f t="shared" si="17"/>
-        <v>6.6031163072794028</v>
+        <f t="shared" si="24"/>
+        <v>5.841738055997463</v>
       </c>
       <c r="U9">
-        <f t="shared" si="17"/>
-        <v>129.9342390029025</v>
+        <f t="shared" si="18"/>
+        <v>128.52828005257157</v>
       </c>
       <c r="V9">
         <f t="shared" si="13"/>
@@ -16585,11 +16585,11 @@
         <v>9.7717853695397216E-3</v>
       </c>
       <c r="Z9">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.2</v>
       </c>
       <c r="AA9">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.13750000000000001</v>
       </c>
       <c r="AB9">
@@ -16600,18 +16600,18 @@
       </c>
       <c r="AD9">
         <f t="shared" si="5"/>
-        <v>25.986847800580502</v>
+        <v>25.705656010514318</v>
       </c>
       <c r="AE9">
         <f t="shared" si="6"/>
-        <v>9.7377269970974965</v>
+        <v>11.143685947428423</v>
       </c>
       <c r="AF9">
         <f t="shared" si="7"/>
         <v>8.0840134650000017</v>
       </c>
       <c r="AG9">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>9.6629351999999997</v>
       </c>
       <c r="AH9">
@@ -16620,7 +16620,7 @@
       </c>
       <c r="AI9">
         <f t="shared" si="9"/>
-        <v>103.947391202322</v>
+        <v>102.82262404205726</v>
       </c>
       <c r="AJ9">
         <f t="shared" si="10"/>
@@ -16693,31 +16693,31 @@
       </c>
       <c r="O10">
         <f t="shared" si="15"/>
-        <v>3.7458961246179854</v>
+        <v>4.544047878107115</v>
       </c>
       <c r="P10">
         <f t="shared" si="15"/>
-        <v>0.27795411564241057</v>
+        <v>1.2089295986534427</v>
       </c>
       <c r="Q10">
         <f t="shared" si="15"/>
-        <v>12.151831204920938</v>
+        <v>13.880958441421086</v>
       </c>
       <c r="R10">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>88.452731035339468</v>
       </c>
       <c r="S10">
-        <f t="shared" si="17"/>
-        <v>34.008487875382016</v>
+        <f t="shared" si="23"/>
+        <v>33.210336121892887</v>
       </c>
       <c r="T10">
-        <f t="shared" si="17"/>
-        <v>6.5565418843575891</v>
+        <f t="shared" si="24"/>
+        <v>5.6255664013465569</v>
       </c>
       <c r="U10">
-        <f t="shared" si="17"/>
-        <v>129.01776079507906</v>
+        <f t="shared" si="18"/>
+        <v>127.28863355857891</v>
       </c>
       <c r="V10">
         <f t="shared" si="13"/>
@@ -16736,11 +16736,11 @@
         <v>9.7617773266647171E-3</v>
       </c>
       <c r="Z10">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.24000000000000002</v>
       </c>
       <c r="AA10">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.16500000000000001</v>
       </c>
       <c r="AB10">
@@ -16751,18 +16751,18 @@
       </c>
       <c r="AD10">
         <f t="shared" si="5"/>
-        <v>30.964262590818976</v>
+        <v>30.549272054058939</v>
       </c>
       <c r="AE10">
         <f t="shared" si="6"/>
-        <v>12.151831204920938</v>
+        <v>13.880958441421086</v>
       </c>
       <c r="AF10">
         <f t="shared" si="7"/>
         <v>9.5375201129999994</v>
       </c>
       <c r="AG10">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>11.6158296</v>
       </c>
       <c r="AH10">
@@ -16771,7 +16771,7 @@
       </c>
       <c r="AI10">
         <f t="shared" si="9"/>
-        <v>98.05349820426008</v>
+        <v>96.739361504519962</v>
       </c>
       <c r="AJ10">
         <f t="shared" si="10"/>
@@ -16844,31 +16844,31 @@
       </c>
       <c r="O11">
         <f t="shared" si="15"/>
-        <v>4.4600876051533334</v>
+        <v>5.408867988081802</v>
       </c>
       <c r="P11">
         <f t="shared" si="15"/>
-        <v>0.33423103051294145</v>
+        <v>1.4271328901308271</v>
       </c>
       <c r="Q11">
         <f t="shared" si="15"/>
-        <v>14.507801125025765</v>
+        <v>16.549483367572094</v>
       </c>
       <c r="R11">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>87.828838510640523</v>
       </c>
       <c r="S11">
-        <f t="shared" si="17"/>
-        <v>33.76861239484667</v>
+        <f t="shared" si="23"/>
+        <v>32.819832011918201</v>
       </c>
       <c r="T11">
-        <f t="shared" si="17"/>
-        <v>6.5102959694870588</v>
+        <f t="shared" si="24"/>
+        <v>5.4173941098691731</v>
       </c>
       <c r="U11">
-        <f t="shared" si="17"/>
-        <v>128.10774687497423</v>
+        <f t="shared" si="18"/>
+        <v>126.0660646324279</v>
       </c>
       <c r="V11">
         <f t="shared" si="13"/>
@@ -16887,11 +16887,11 @@
         <v>9.7520725620833561E-3</v>
       </c>
       <c r="Z11">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.28000000000000003</v>
       </c>
       <c r="AA11">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.1925</v>
       </c>
       <c r="AB11">
@@ -16902,18 +16902,18 @@
       </c>
       <c r="AD11">
         <f t="shared" si="5"/>
-        <v>35.870169124992785</v>
+        <v>35.298498097079815</v>
       </c>
       <c r="AE11">
         <f t="shared" si="6"/>
-        <v>14.507801125025765</v>
+        <v>16.549483367572094</v>
       </c>
       <c r="AF11">
         <f t="shared" si="7"/>
         <v>10.934131361999999</v>
       </c>
       <c r="AG11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>13.591124999999998</v>
       </c>
       <c r="AH11">
@@ -16922,7 +16922,7 @@
       </c>
       <c r="AI11">
         <f t="shared" si="9"/>
-        <v>92.23757774998144</v>
+        <v>90.767566535348081</v>
       </c>
       <c r="AJ11">
         <f t="shared" si="10"/>
@@ -16995,31 +16995,31 @@
       </c>
       <c r="O12">
         <f t="shared" si="15"/>
-        <v>5.1394791478885296</v>
+        <v>6.2359883510971201</v>
       </c>
       <c r="P12">
         <f t="shared" si="15"/>
-        <v>0.38802075443099504</v>
+        <v>1.6354718323190491</v>
       </c>
       <c r="Q12">
         <f t="shared" si="15"/>
-        <v>16.793553352621274</v>
+        <v>19.137513633717873</v>
       </c>
       <c r="R12">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>87.209346549698282</v>
       </c>
       <c r="S12">
-        <f t="shared" si="17"/>
-        <v>33.53042885211147</v>
+        <f t="shared" si="23"/>
+        <v>32.433919648902879</v>
       </c>
       <c r="T12">
-        <f t="shared" si="17"/>
-        <v>6.4643762455690048</v>
+        <f t="shared" si="24"/>
+        <v>5.2169251676809507</v>
       </c>
       <c r="U12">
-        <f t="shared" si="17"/>
-        <v>127.20415164737872</v>
+        <f t="shared" si="18"/>
+        <v>124.86019136628212</v>
       </c>
       <c r="V12">
         <f t="shared" si="13"/>
@@ -17038,11 +17038,11 @@
         <v>9.7422228739226183E-3</v>
       </c>
       <c r="Z12">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.32</v>
       </c>
       <c r="AA12">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.22</v>
       </c>
       <c r="AB12">
@@ -17053,18 +17053,18 @@
       </c>
       <c r="AD12">
         <f t="shared" si="5"/>
-        <v>40.705328527161193</v>
+        <v>39.95526123721028</v>
       </c>
       <c r="AE12">
         <f t="shared" si="6"/>
-        <v>16.793553352621274</v>
+        <v>19.137513633717873</v>
       </c>
       <c r="AF12">
         <f t="shared" si="7"/>
         <v>12.272719799999999</v>
       </c>
       <c r="AG12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>15.584098199999998</v>
       </c>
       <c r="AH12">
@@ -17073,7 +17073,7 @@
       </c>
       <c r="AI12">
         <f t="shared" si="9"/>
-        <v>86.498823120217537</v>
+        <v>84.904930129071843</v>
       </c>
       <c r="AJ12">
         <f t="shared" si="10"/>
@@ -17146,31 +17146,31 @@
       </c>
       <c r="O13">
         <f t="shared" si="15"/>
-        <v>5.8028466867382704</v>
+        <v>7.0442269592612305</v>
       </c>
       <c r="P13">
         <f t="shared" si="15"/>
-        <v>0.43936758815195276</v>
+        <v>1.8342734852030365</v>
       </c>
       <c r="Q13">
         <f t="shared" si="15"/>
-        <v>19.050574161315495</v>
+        <v>21.686860330889502</v>
       </c>
       <c r="R13">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>86.594224113574768</v>
       </c>
       <c r="S13">
-        <f t="shared" si="17"/>
-        <v>33.293925313261731</v>
+        <f t="shared" si="23"/>
+        <v>32.052545040738771</v>
       </c>
       <c r="T13">
-        <f t="shared" si="17"/>
-        <v>6.4187804118480472</v>
+        <f t="shared" si="24"/>
+        <v>5.0238745147969635</v>
       </c>
       <c r="U13">
-        <f t="shared" si="17"/>
-        <v>126.30692983868451</v>
+        <f t="shared" si="18"/>
+        <v>123.6706436691105</v>
       </c>
       <c r="V13">
         <f t="shared" si="13"/>
@@ -17189,11 +17189,11 @@
         <v>9.732071585767034E-3</v>
       </c>
       <c r="Z13">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.36</v>
       </c>
       <c r="AA13">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.2475</v>
       </c>
       <c r="AB13">
@@ -17204,18 +17204,18 @@
       </c>
       <c r="AD13">
         <f t="shared" si="5"/>
-        <v>45.470494741926423</v>
+        <v>44.521431720879782</v>
       </c>
       <c r="AE13">
         <f t="shared" si="6"/>
-        <v>19.050574161315495</v>
+        <v>21.686860330889502</v>
       </c>
       <c r="AF13">
         <f t="shared" si="7"/>
         <v>13.552138660499999</v>
       </c>
       <c r="AG13">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>17.586227399999999</v>
       </c>
       <c r="AH13">
@@ -17224,7 +17224,7 @@
       </c>
       <c r="AI13">
         <f t="shared" si="9"/>
-        <v>80.836435096758095</v>
+        <v>79.149211948230715</v>
       </c>
       <c r="AJ13">
         <f t="shared" si="10"/>
@@ -17297,31 +17297,31 @@
       </c>
       <c r="O14">
         <f t="shared" si="15"/>
-        <v>6.4486020714425578</v>
+        <v>7.8320371698154645</v>
       </c>
       <c r="P14">
         <f t="shared" si="15"/>
-        <v>0.49046281620304644</v>
+        <v>2.0260013602138409</v>
       </c>
       <c r="Q14">
         <f t="shared" si="15"/>
-        <v>21.270089505383581</v>
+        <v>24.189063147767243</v>
       </c>
       <c r="R14">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>85.98344038226206</v>
       </c>
       <c r="S14">
-        <f t="shared" si="17"/>
-        <v>33.059089928557441</v>
+        <f t="shared" si="23"/>
+        <v>31.675654830184534</v>
       </c>
       <c r="T14">
-        <f t="shared" si="17"/>
-        <v>6.3735061837969536</v>
+        <f t="shared" si="24"/>
+        <v>4.8379676397861591</v>
       </c>
       <c r="U14">
-        <f t="shared" si="17"/>
-        <v>125.41603649461642</v>
+        <f t="shared" si="18"/>
+        <v>122.49706285223276</v>
       </c>
       <c r="V14">
         <f t="shared" si="13"/>
@@ -17340,11 +17340,11 @@
         <v>9.7221785027928834E-3</v>
       </c>
       <c r="Z14">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.39999999999999997</v>
       </c>
       <c r="AA14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.27500000000000002</v>
       </c>
       <c r="AB14">
@@ -17355,18 +17355,18 @@
       </c>
       <c r="AD14">
         <f t="shared" si="5"/>
-        <v>50.166414597846561</v>
+        <v>48.998825140893096</v>
       </c>
       <c r="AE14">
         <f t="shared" si="6"/>
-        <v>21.270089505383581</v>
+        <v>24.189063147767243</v>
       </c>
       <c r="AF14">
         <f t="shared" si="7"/>
         <v>14.771232134999998</v>
       </c>
       <c r="AG14">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>19.587781799999998</v>
       </c>
       <c r="AH14">
@@ -17375,7 +17375,7 @@
       </c>
       <c r="AI14">
         <f t="shared" si="9"/>
-        <v>75.249621896769867</v>
+        <v>73.498237711339669</v>
       </c>
       <c r="AJ14">
         <f t="shared" si="10"/>
@@ -17448,31 +17448,31 @@
       </c>
       <c r="O15">
         <f t="shared" si="15"/>
-        <v>7.0618370681604432</v>
+        <v>8.5845517125994526</v>
       </c>
       <c r="P15">
         <f t="shared" si="15"/>
-        <v>0.54020570699782233</v>
+        <v>2.2098168105745088</v>
       </c>
       <c r="Q15">
         <f t="shared" si="15"/>
-        <v>23.426470022020212</v>
+        <v>26.61879577003586</v>
       </c>
       <c r="R15">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>85.376964753138097</v>
       </c>
       <c r="S15">
-        <f t="shared" si="17"/>
-        <v>32.825910931839559</v>
+        <f t="shared" si="23"/>
+        <v>31.303196287400549</v>
       </c>
       <c r="T15">
-        <f t="shared" si="17"/>
-        <v>6.3285512930021772</v>
+        <f t="shared" si="24"/>
+        <v>4.6589401894254907</v>
       </c>
       <c r="U15">
-        <f t="shared" si="17"/>
-        <v>124.53142697797979</v>
+        <f t="shared" si="18"/>
+        <v>121.33910122996414</v>
       </c>
       <c r="V15">
         <f t="shared" si="13"/>
@@ -17491,11 +17491,11 @@
         <v>9.712294236529492E-3</v>
       </c>
       <c r="Z15">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.43999999999999995</v>
       </c>
       <c r="AA15">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.30250000000000005</v>
       </c>
       <c r="AB15">
@@ -17506,18 +17506,18 @@
       </c>
       <c r="AD15">
         <f t="shared" si="5"/>
-        <v>54.793827870311098</v>
+        <v>53.389204541184213</v>
       </c>
       <c r="AE15">
         <f t="shared" si="6"/>
-        <v>23.426470022020212</v>
+        <v>26.61879577003586</v>
       </c>
       <c r="AF15">
         <f t="shared" si="7"/>
         <v>15.928864347000003</v>
       </c>
       <c r="AG15">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>21.583927199999998</v>
       </c>
       <c r="AH15">
@@ -17526,7 +17526,7 @@
       </c>
       <c r="AI15">
         <f t="shared" si="9"/>
-        <v>69.7375991076687</v>
+        <v>67.94989668877993</v>
       </c>
       <c r="AJ15">
         <f t="shared" si="10"/>
@@ -17599,31 +17599,31 @@
       </c>
       <c r="O16">
         <f t="shared" si="15"/>
-        <v>7.6500513600595283</v>
+        <v>9.3093106974283906</v>
       </c>
       <c r="P16">
         <f t="shared" si="15"/>
-        <v>0.58876751294979979</v>
+        <v>2.3861434072013363</v>
       </c>
       <c r="Q16">
         <f t="shared" si="15"/>
-        <v>25.527244033576011</v>
+        <v>28.98387926519635</v>
       </c>
       <c r="R16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>84.774766839433354</v>
       </c>
       <c r="S16">
-        <f t="shared" si="17"/>
-        <v>32.594376639940471</v>
+        <f t="shared" si="23"/>
+        <v>30.935117302571609</v>
       </c>
       <c r="T16">
-        <f t="shared" si="17"/>
-        <v>6.2839134870502003</v>
+        <f t="shared" si="24"/>
+        <v>4.4865375927986637</v>
       </c>
       <c r="U16">
-        <f t="shared" si="17"/>
-        <v>123.65305696642397</v>
+        <f t="shared" si="18"/>
+        <v>120.19642173480364</v>
       </c>
       <c r="V16">
         <f t="shared" si="13"/>
@@ -17642,11 +17642,11 @@
         <v>9.7025443249506727E-3</v>
       </c>
       <c r="Z16">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.47999999999999993</v>
       </c>
       <c r="AA16">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.33000000000000007</v>
       </c>
       <c r="AB16">
@@ -17657,18 +17657,18 @@
       </c>
       <c r="AD16">
         <f t="shared" si="5"/>
-        <v>59.353467343883501</v>
+        <v>57.694282432705734</v>
       </c>
       <c r="AE16">
         <f t="shared" si="6"/>
-        <v>25.527244033576011</v>
+        <v>28.98387926519635</v>
       </c>
       <c r="AF16">
         <f t="shared" si="7"/>
         <v>17.023923378000006</v>
       </c>
       <c r="AG16">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>23.576113799999995</v>
       </c>
       <c r="AH16">
@@ -17677,7 +17677,7 @@
       </c>
       <c r="AI16">
         <f t="shared" si="9"/>
-        <v>64.299589622540481</v>
+        <v>62.502139302097902</v>
       </c>
       <c r="AJ16">
         <f t="shared" si="10"/>
@@ -17750,31 +17750,31 @@
       </c>
       <c r="O17">
         <f t="shared" si="15"/>
-        <v>8.2155965479013844</v>
+        <v>10.008705621383651</v>
       </c>
       <c r="P17">
         <f t="shared" si="15"/>
-        <v>0.63658247058532069</v>
+        <v>2.5556583006950051</v>
       </c>
       <c r="Q17">
         <f t="shared" si="15"/>
-        <v>27.567538549778391</v>
+        <v>31.279723453370295</v>
       </c>
       <c r="R17">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>84.176816468708367</v>
       </c>
       <c r="S17">
-        <f t="shared" si="17"/>
-        <v>32.364475452098617</v>
+        <f t="shared" si="23"/>
+        <v>30.57136637861635</v>
       </c>
       <c r="T17">
-        <f t="shared" si="17"/>
-        <v>6.239590529414679</v>
+        <f t="shared" si="24"/>
+        <v>4.3205146993049945</v>
       </c>
       <c r="U17">
-        <f t="shared" si="17"/>
-        <v>122.78088245022161</v>
+        <f t="shared" si="18"/>
+        <v>119.06869754662971</v>
       </c>
       <c r="V17">
         <f t="shared" si="13"/>
@@ -17793,11 +17793,11 @@
         <v>9.6931615463480766E-3</v>
       </c>
       <c r="Z17">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.51999999999999991</v>
       </c>
       <c r="AA17">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.3575000000000001</v>
       </c>
       <c r="AB17">
@@ -17808,18 +17808,18 @@
       </c>
       <c r="AD17">
         <f t="shared" si="5"/>
-        <v>63.846058874115229</v>
+        <v>61.915722724247438</v>
       </c>
       <c r="AE17">
         <f t="shared" si="6"/>
-        <v>27.567538549778391</v>
+        <v>31.279723453370295</v>
       </c>
       <c r="AF17">
         <f t="shared" si="7"/>
         <v>18.055318495500003</v>
       </c>
       <c r="AG17">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>25.567232999999995</v>
       </c>
       <c r="AH17">
@@ -17828,7 +17828,7 @@
       </c>
       <c r="AI17">
         <f t="shared" si="9"/>
-        <v>58.934823576106382</v>
+        <v>57.152974822382269</v>
       </c>
       <c r="AJ17">
         <f t="shared" si="10"/>
@@ -17901,31 +17901,31 @@
       </c>
       <c r="O18">
         <f t="shared" si="15"/>
-        <v>8.7614601506227459</v>
+        <v>10.685763376017576</v>
       </c>
       <c r="P18">
         <f t="shared" si="15"/>
-        <v>0.68604880065561424</v>
+        <v>2.7209935699363665</v>
       </c>
       <c r="Q18">
         <f t="shared" si="15"/>
-        <v>29.556817269936445</v>
+        <v>33.516065264611967</v>
       </c>
       <c r="R18">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>83.583083681341975</v>
       </c>
       <c r="S18">
-        <f t="shared" si="17"/>
-        <v>32.136195849377252</v>
+        <f t="shared" si="23"/>
+        <v>30.211892623982422</v>
       </c>
       <c r="T18">
-        <f t="shared" si="17"/>
-        <v>6.195580199344386</v>
+        <f t="shared" si="24"/>
+        <v>4.1606354300636337</v>
       </c>
       <c r="U18">
-        <f t="shared" si="17"/>
-        <v>121.91485973006355</v>
+        <f t="shared" si="18"/>
+        <v>117.95561173538803</v>
       </c>
       <c r="V18">
         <f t="shared" si="13"/>
@@ -17944,11 +17944,11 @@
         <v>9.6845299295162945E-3</v>
       </c>
       <c r="Z18">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.55999999999999994</v>
       </c>
       <c r="AA18">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.38500000000000012</v>
       </c>
       <c r="AB18">
@@ -17959,18 +17959,18 @@
       </c>
       <c r="AD18">
         <f t="shared" si="5"/>
-        <v>68.272321448835584</v>
+        <v>66.055142571817285</v>
       </c>
       <c r="AE18">
         <f t="shared" si="6"/>
-        <v>29.556817269936445</v>
+        <v>33.516065264611967</v>
       </c>
       <c r="AF18">
         <f t="shared" si="7"/>
         <v>19.021968735000012</v>
       </c>
       <c r="AG18">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>27.560416199999995</v>
       </c>
       <c r="AH18">
@@ -17979,7 +17979,7 @@
       </c>
       <c r="AI18">
         <f t="shared" si="9"/>
-        <v>53.642538281227971</v>
+        <v>51.900469163570747</v>
       </c>
       <c r="AJ18">
         <f t="shared" si="10"/>
@@ -18052,31 +18052,31 @@
       </c>
       <c r="O19">
         <f t="shared" si="15"/>
-        <v>9.2838816059126827</v>
+        <v>11.336762254473637</v>
       </c>
       <c r="P19">
         <f t="shared" si="15"/>
-        <v>0.73612870824806009</v>
+        <v>2.8813365577825358</v>
       </c>
       <c r="Q19">
         <f t="shared" si="15"/>
-        <v>31.487359585130605</v>
+        <v>35.685448083225978</v>
       </c>
       <c r="R19">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>82.993538729030192</v>
       </c>
       <c r="S19">
-        <f t="shared" si="17"/>
-        <v>31.909526394087315</v>
+        <f t="shared" si="23"/>
+        <v>29.856645745526361</v>
       </c>
       <c r="T19">
-        <f t="shared" si="17"/>
-        <v>6.1518802917519402</v>
+        <f t="shared" si="24"/>
+        <v>4.0066724422174644</v>
       </c>
       <c r="U19">
-        <f t="shared" si="17"/>
-        <v>121.05494541486939</v>
+        <f t="shared" si="18"/>
+        <v>116.85685691677402</v>
       </c>
       <c r="V19">
         <f t="shared" si="13"/>
@@ -18095,11 +18095,11 @@
         <v>9.6764382340940053E-3</v>
       </c>
       <c r="Z19">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.6</v>
       </c>
       <c r="AA19">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.41250000000000014</v>
       </c>
       <c r="AB19">
@@ -18110,18 +18110,18 @@
       </c>
       <c r="AD19">
         <f t="shared" si="5"/>
-        <v>72.632967248921631</v>
+        <v>70.11411415006441</v>
       </c>
       <c r="AE19">
         <f t="shared" si="6"/>
-        <v>31.487359585130605</v>
+        <v>35.685448083225978</v>
       </c>
       <c r="AF19">
         <f t="shared" si="7"/>
         <v>19.922811232500006</v>
       </c>
       <c r="AG19">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>29.558776199999993</v>
       </c>
       <c r="AH19">
@@ -18130,7 +18130,7 @@
       </c>
       <c r="AI19">
         <f t="shared" si="9"/>
-        <v>48.421978165947763</v>
+        <v>46.742742766709611</v>
       </c>
       <c r="AJ19">
         <f t="shared" si="10"/>
@@ -18203,42 +18203,42 @@
       </c>
       <c r="O20">
         <f t="shared" si="15"/>
-        <v>9.7879402707856684</v>
+        <v>11.966819958522809</v>
       </c>
       <c r="P20">
         <f t="shared" si="15"/>
-        <v>0.78588338289667359</v>
+        <v>3.0359651943406685</v>
       </c>
       <c r="Q20">
         <f t="shared" si="15"/>
-        <v>33.374343580386622</v>
+        <v>37.803305079567693</v>
       </c>
       <c r="R20">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>82.408152073295767</v>
       </c>
       <c r="S20">
-        <f t="shared" si="17"/>
-        <v>31.684455729214335</v>
+        <f t="shared" si="23"/>
+        <v>29.505576041477195</v>
       </c>
       <c r="T20">
-        <f t="shared" si="17"/>
-        <v>6.1084886171033261</v>
+        <f t="shared" si="24"/>
+        <v>3.8584068056593313</v>
       </c>
       <c r="U20">
-        <f t="shared" si="17"/>
-        <v>120.20109641961336</v>
+        <f t="shared" si="18"/>
+        <v>115.77213492043229</v>
       </c>
       <c r="V20">
-        <f t="shared" ref="V20:X28" si="21">V19</f>
+        <f t="shared" ref="V20:X28" si="25">V19</f>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X20">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y20">
@@ -18246,11 +18246,11 @@
         <v>9.6685808399261282E-3</v>
       </c>
       <c r="Z20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.64</v>
       </c>
       <c r="AA20">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.44000000000000017</v>
       </c>
       <c r="AB20">
@@ -18261,18 +18261,18 @@
       </c>
       <c r="AD20">
         <f t="shared" si="5"/>
-        <v>76.928701708552552</v>
+        <v>74.094166349076673</v>
       </c>
       <c r="AE20">
         <f t="shared" si="6"/>
-        <v>33.374343580386622</v>
+        <v>37.803305079567693</v>
       </c>
       <c r="AF20">
         <f t="shared" si="7"/>
         <v>20.75678352000001</v>
       </c>
       <c r="AG20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>31.564285799999993</v>
       </c>
       <c r="AH20">
@@ -18281,7 +18281,7 @@
       </c>
       <c r="AI20">
         <f t="shared" si="9"/>
-        <v>43.272394711060812</v>
+        <v>41.67796857135562</v>
       </c>
       <c r="AJ20">
         <f t="shared" si="10"/>
@@ -18354,42 +18354,42 @@
       </c>
       <c r="O21">
         <f t="shared" si="15"/>
-        <v>10.281639422150587</v>
+        <v>12.583977605517216</v>
       </c>
       <c r="P21">
         <f t="shared" si="15"/>
-        <v>0.83432799869181284</v>
+        <v>3.1841033082790937</v>
       </c>
       <c r="Q21">
         <f t="shared" si="15"/>
-        <v>35.212817036834352</v>
+        <v>39.864930529788182</v>
       </c>
       <c r="R21">
-        <f t="shared" si="17"/>
+        <f t="shared" si="22"/>
         <v>81.826894384008128</v>
       </c>
       <c r="S21">
-        <f t="shared" si="17"/>
-        <v>31.460972577849414</v>
+        <f t="shared" si="23"/>
+        <v>29.158634394482785</v>
       </c>
       <c r="T21">
-        <f t="shared" si="17"/>
-        <v>6.0654030013081872</v>
+        <f t="shared" si="24"/>
+        <v>3.7156276917209063</v>
       </c>
       <c r="U21">
-        <f t="shared" si="17"/>
-        <v>119.35326996316566</v>
+        <f t="shared" si="18"/>
+        <v>114.70115647021183</v>
       </c>
       <c r="V21">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W21">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X21">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y21">
@@ -18397,11 +18397,11 @@
         <v>9.6610836225848387E-3</v>
       </c>
       <c r="Z21">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.68</v>
       </c>
       <c r="AA21">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.46750000000000019</v>
       </c>
       <c r="AB21">
@@ -18412,18 +18412,18 @@
       </c>
       <c r="AD21">
         <f t="shared" si="5"/>
-        <v>81.160223574952653</v>
+        <v>77.996786399744053</v>
       </c>
       <c r="AE21">
         <f t="shared" si="6"/>
-        <v>35.212817036834352</v>
+        <v>39.864930529788182</v>
       </c>
       <c r="AF21">
         <f t="shared" si="7"/>
         <v>21.522844662000008</v>
       </c>
       <c r="AG21">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>33.578770199999994</v>
       </c>
       <c r="AH21">
@@ -18432,7 +18432,7 @@
       </c>
       <c r="AI21">
         <f t="shared" si="9"/>
-        <v>38.193046388213006</v>
+        <v>36.704370070467775</v>
       </c>
       <c r="AJ21">
         <f t="shared" si="10"/>
@@ -18505,42 +18505,42 @@
       </c>
       <c r="O22">
         <f t="shared" si="15"/>
-        <v>10.774494257375792</v>
+        <v>13.197787735262068</v>
       </c>
       <c r="P22">
         <f t="shared" si="15"/>
-        <v>0.88231671438910197</v>
+        <v>3.3268059266184693</v>
       </c>
       <c r="Q22">
         <f t="shared" si="15"/>
-        <v>37.024810433851115</v>
+        <v>41.892593123966705</v>
       </c>
       <c r="R22">
-        <f t="shared" ref="R22:U28" si="22">R21*(1-$V21)</f>
+        <f t="shared" si="22"/>
         <v>81.249736537913847</v>
       </c>
       <c r="S22">
-        <f t="shared" si="22"/>
-        <v>31.239065742624206</v>
+        <f t="shared" si="23"/>
+        <v>28.81577226473793</v>
       </c>
       <c r="T22">
-        <f t="shared" si="22"/>
-        <v>6.0226212856108976</v>
+        <f t="shared" si="24"/>
+        <v>3.5781320733815303</v>
       </c>
       <c r="U22">
-        <f t="shared" si="22"/>
-        <v>118.51142356614889</v>
+        <f t="shared" si="18"/>
+        <v>113.6436408760333</v>
       </c>
       <c r="V22">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W22">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X22">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y22">
@@ -18548,11 +18548,11 @@
         <v>9.6540174916241988E-3</v>
       </c>
       <c r="Z22">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.72000000000000008</v>
       </c>
       <c r="AA22">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.49500000000000022</v>
       </c>
       <c r="AB22">
@@ -18563,18 +18563,18 @@
       </c>
       <c r="AD22">
         <f t="shared" si="5"/>
-        <v>85.328224967627207</v>
+        <v>81.823421430743991</v>
       </c>
       <c r="AE22">
         <f t="shared" si="6"/>
-        <v>37.024810433851115</v>
+        <v>41.892593123966705</v>
       </c>
       <c r="AF22">
         <f t="shared" si="7"/>
         <v>22.21993293300001</v>
       </c>
       <c r="AG22">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>35.60446559999999</v>
       </c>
       <c r="AH22">
@@ -18583,7 +18583,7 @@
       </c>
       <c r="AI22">
         <f t="shared" si="9"/>
-        <v>33.183198598521685</v>
+        <v>31.820219445289311</v>
       </c>
       <c r="AJ22">
         <f t="shared" si="10"/>
@@ -18656,42 +18656,42 @@
       </c>
       <c r="O23">
         <f t="shared" si="15"/>
-        <v>11.265843894850111</v>
+        <v>13.807626316806733</v>
       </c>
       <c r="P23">
         <f t="shared" si="15"/>
-        <v>0.93027667351760179</v>
+        <v>3.4646935634292735</v>
       </c>
       <c r="Q23">
         <f t="shared" si="15"/>
-        <v>38.830149951190265</v>
+        <v>43.906349263058488</v>
       </c>
       <c r="R23">
         <f t="shared" si="22"/>
         <v>80.676649617177503</v>
       </c>
       <c r="S23">
-        <f t="shared" si="22"/>
-        <v>31.018724105149889</v>
+        <f t="shared" si="23"/>
+        <v>28.476941683193267</v>
       </c>
       <c r="T23">
-        <f t="shared" si="22"/>
-        <v>5.9801413264823982</v>
+        <f t="shared" si="24"/>
+        <v>3.4457244365707265</v>
       </c>
       <c r="U23">
-        <f t="shared" si="22"/>
-        <v>117.67551504880973</v>
+        <f t="shared" si="18"/>
+        <v>112.59931573694151</v>
       </c>
       <c r="V23">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W23">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X23">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y23">
@@ -18699,11 +18699,11 @@
         <v>9.6471049232439137E-3</v>
       </c>
       <c r="Z23">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.76000000000000012</v>
       </c>
       <c r="AA23">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.52250000000000019</v>
       </c>
       <c r="AB23">
@@ -18714,18 +18714,18 @@
       </c>
       <c r="AD23">
         <f t="shared" si="5"/>
-        <v>89.433391437095409</v>
+        <v>85.575479960075555</v>
       </c>
       <c r="AE23">
         <f t="shared" si="6"/>
-        <v>38.830149951190265</v>
+        <v>43.906349263058488</v>
       </c>
       <c r="AF23">
         <f t="shared" si="7"/>
         <v>22.847006589000014</v>
       </c>
       <c r="AG23">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>37.643471399999989</v>
       </c>
       <c r="AH23">
@@ -18734,7 +18734,7 @@
       </c>
       <c r="AI23">
         <f t="shared" si="9"/>
-        <v>28.24212361171432</v>
+        <v>27.023835776865951</v>
       </c>
       <c r="AJ23">
         <f t="shared" si="10"/>
@@ -18807,42 +18807,42 @@
       </c>
       <c r="O24">
         <f t="shared" si="15"/>
-        <v>11.755187374539915</v>
+        <v>14.413028755155956</v>
       </c>
       <c r="P24">
         <f t="shared" si="15"/>
-        <v>0.97612100448720085</v>
+        <v>3.5958654978461255</v>
       </c>
       <c r="Q24">
         <f t="shared" si="15"/>
-        <v>40.623567471094461</v>
+        <v>45.901153345069361</v>
       </c>
       <c r="R24">
         <f t="shared" si="22"/>
         <v>80.107604907932711</v>
       </c>
       <c r="S24">
-        <f t="shared" si="22"/>
-        <v>30.799936625460084</v>
+        <f t="shared" si="23"/>
+        <v>28.142095244844043</v>
       </c>
       <c r="T24">
-        <f t="shared" si="22"/>
-        <v>5.9379609955127988</v>
+        <f t="shared" si="24"/>
+        <v>3.3182165021538741</v>
       </c>
       <c r="U24">
-        <f t="shared" si="22"/>
-        <v>116.84550252890553</v>
+        <f t="shared" si="18"/>
+        <v>111.56791665493063</v>
       </c>
       <c r="V24">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W24">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X24">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y24">
@@ -18850,11 +18850,11 @@
         <v>9.6400174518286204E-3</v>
       </c>
       <c r="Z24">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.8</v>
       </c>
       <c r="AA24">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="AB24">
@@ -18865,18 +18865,18 @@
       </c>
       <c r="AD24">
         <f t="shared" si="5"/>
-        <v>93.476402023124422</v>
+        <v>89.254333323944508</v>
       </c>
       <c r="AE24">
         <f t="shared" si="6"/>
-        <v>40.623567471094461</v>
+        <v>45.901153345069361</v>
       </c>
       <c r="AF24">
         <f t="shared" si="7"/>
         <v>23.402998740000008</v>
       </c>
       <c r="AG24">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>39.69773519999999</v>
       </c>
       <c r="AH24">
@@ -18885,7 +18885,7 @@
       </c>
       <c r="AI24">
         <f t="shared" si="9"/>
-        <v>23.369100505781105</v>
+        <v>22.31358333098612</v>
       </c>
       <c r="AJ24">
         <f t="shared" si="10"/>
@@ -18958,42 +18958,42 @@
       </c>
       <c r="O25">
         <f t="shared" si="15"/>
-        <v>12.241251658542275</v>
+        <v>15.012757897902212</v>
       </c>
       <c r="P25">
         <f t="shared" si="15"/>
-        <v>1.0211668206952647</v>
+        <v>3.7218180417942874</v>
       </c>
       <c r="Q25">
         <f t="shared" si="15"/>
-        <v>42.405820580394121</v>
+        <v>47.877978040853023</v>
       </c>
       <c r="R25">
         <f t="shared" si="22"/>
         <v>79.542573898843486</v>
       </c>
       <c r="S25">
-        <f t="shared" si="22"/>
-        <v>30.582692341457722</v>
+        <f t="shared" si="23"/>
+        <v>27.811186102097786</v>
       </c>
       <c r="T25">
-        <f t="shared" si="22"/>
-        <v>5.8960781793047357</v>
+        <f t="shared" si="24"/>
+        <v>3.1954269582057129</v>
       </c>
       <c r="U25">
-        <f t="shared" si="22"/>
-        <v>116.02134441960588</v>
+        <f t="shared" si="18"/>
+        <v>110.54918695914698</v>
       </c>
       <c r="V25">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W25">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X25">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y25">
@@ -19001,11 +19001,11 @@
         <v>9.6329564083451318E-3</v>
       </c>
       <c r="Z25">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.8</v>
       </c>
       <c r="AA25">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="AB25">
@@ -19016,18 +19016,18 @@
       </c>
       <c r="AD25">
         <f t="shared" si="5"/>
-        <v>92.817075535684708</v>
+        <v>88.439349567317592</v>
       </c>
       <c r="AE25">
         <f t="shared" si="6"/>
-        <v>42.405820580394121</v>
+        <v>47.877978040853023</v>
       </c>
       <c r="AF25">
         <f t="shared" si="7"/>
         <v>22.749390510000008</v>
       </c>
       <c r="AG25">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>41.768855999999992</v>
       </c>
       <c r="AH25">
@@ -19036,7 +19036,7 @@
       </c>
       <c r="AI25">
         <f t="shared" si="9"/>
-        <v>23.204268883921173</v>
+        <v>22.109837391829387</v>
       </c>
       <c r="AJ25">
         <f t="shared" si="10"/>
@@ -19109,42 +19109,42 @@
       </c>
       <c r="O26">
         <f t="shared" si="15"/>
-        <v>12.726615631634211</v>
+        <v>15.609428041780035</v>
       </c>
       <c r="P26">
         <f t="shared" si="15"/>
-        <v>1.0657322206325155</v>
+        <v>3.8430417978090174</v>
       </c>
       <c r="Q26">
         <f t="shared" si="15"/>
-        <v>44.180715572591069</v>
+        <v>49.840837559913325</v>
       </c>
       <c r="R26">
         <f t="shared" si="22"/>
         <v>78.981528279675715</v>
       </c>
       <c r="S26">
-        <f t="shared" si="22"/>
-        <v>30.366980368365788</v>
+        <f t="shared" si="23"/>
+        <v>27.484167958219963</v>
       </c>
       <c r="T26">
-        <f t="shared" si="22"/>
-        <v>5.8544907793674845</v>
+        <f t="shared" si="24"/>
+        <v>3.0771812021909826</v>
       </c>
       <c r="U26">
-        <f t="shared" si="22"/>
-        <v>115.20299942740893</v>
+        <f t="shared" si="18"/>
+        <v>109.54287744008667</v>
       </c>
       <c r="V26">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W26">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X26">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y26">
@@ -19152,11 +19152,11 @@
         <v>9.625994989035767E-3</v>
       </c>
       <c r="Z26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.8</v>
       </c>
       <c r="AA26">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="AB26">
@@ -19167,18 +19167,18 @@
       </c>
       <c r="AD26">
         <f t="shared" si="5"/>
-        <v>92.162399541927144</v>
+        <v>87.634301952069336</v>
       </c>
       <c r="AE26">
         <f t="shared" si="6"/>
-        <v>44.180715572591069</v>
+        <v>49.840837559913325</v>
       </c>
       <c r="AF26">
         <f t="shared" si="7"/>
         <v>22.088643059999999</v>
       </c>
       <c r="AG26">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>43.857791399999996</v>
       </c>
       <c r="AH26">
@@ -19187,7 +19187,7 @@
       </c>
       <c r="AI26">
         <f t="shared" si="9"/>
-        <v>23.040599885481782</v>
+        <v>21.908575488017334</v>
       </c>
       <c r="AJ26">
         <f t="shared" si="10"/>
@@ -19260,42 +19260,42 @@
       </c>
       <c r="O27">
         <f t="shared" si="15"/>
-        <v>13.212754101818039</v>
+        <v>16.204548939143283</v>
       </c>
       <c r="P27">
         <f t="shared" si="15"/>
-        <v>1.1122282879881853</v>
+        <v>3.9621139073144165</v>
       </c>
       <c r="Q27">
         <f t="shared" si="15"/>
-        <v>45.955662449927573</v>
+        <v>51.79734290657899</v>
       </c>
       <c r="R27">
         <f t="shared" si="22"/>
         <v>78.42443993987871</v>
       </c>
       <c r="S27">
-        <f t="shared" si="22"/>
-        <v>30.152789898181961</v>
+        <f t="shared" si="23"/>
+        <v>27.160995060856717</v>
       </c>
       <c r="T27">
-        <f t="shared" si="22"/>
-        <v>5.8131967120118144</v>
+        <f t="shared" si="24"/>
+        <v>2.9633110926855832</v>
       </c>
       <c r="U27">
-        <f t="shared" si="22"/>
-        <v>114.39042655007243</v>
+        <f t="shared" si="18"/>
+        <v>108.54874609342102</v>
       </c>
       <c r="V27">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W27">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X27">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y27">
@@ -19303,11 +19303,11 @@
         <v>9.6195062362388964E-3</v>
       </c>
       <c r="Z27">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.8</v>
       </c>
       <c r="AA27">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="AB27">
@@ -19318,18 +19318,18 @@
       </c>
       <c r="AD27">
         <f t="shared" si="5"/>
-        <v>91.51234124005795</v>
+        <v>86.838996874736821</v>
       </c>
       <c r="AE27">
         <f t="shared" si="6"/>
-        <v>45.955662449927573</v>
+        <v>51.79734290657899</v>
       </c>
       <c r="AF27">
         <f t="shared" si="7"/>
         <v>21.420751770000003</v>
       </c>
       <c r="AG27">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>45.964943399999996</v>
       </c>
       <c r="AH27">
@@ -19338,7 +19338,7 @@
       </c>
       <c r="AI27">
         <f t="shared" si="9"/>
-        <v>22.878085310014484</v>
+        <v>21.709749218684195</v>
       </c>
       <c r="AJ27">
         <f t="shared" si="10"/>
@@ -19411,42 +19411,42 @@
       </c>
       <c r="O28">
         <f t="shared" si="15"/>
-        <v>13.699565800862921</v>
+        <v>16.798053804366251</v>
       </c>
       <c r="P28">
         <f t="shared" si="15"/>
-        <v>1.1602770917544101</v>
+        <v>4.0788162897147817</v>
       </c>
       <c r="Q28">
         <f t="shared" si="15"/>
-        <v>47.729905925440633</v>
+        <v>53.746933126904295</v>
       </c>
       <c r="R28">
         <f t="shared" si="22"/>
         <v>77.871280967176745</v>
       </c>
       <c r="S28">
-        <f t="shared" si="22"/>
-        <v>29.940110199137081</v>
+        <f t="shared" si="23"/>
+        <v>26.84162219563375</v>
       </c>
       <c r="T28">
-        <f t="shared" si="22"/>
-        <v>5.7721939082455895</v>
+        <f t="shared" si="24"/>
+        <v>2.8536547102852174</v>
       </c>
       <c r="U28">
-        <f t="shared" si="22"/>
-        <v>113.58358507455937</v>
+        <f t="shared" si="18"/>
+        <v>107.5665578730957</v>
       </c>
       <c r="V28">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>7.0534003574144162E-3</v>
       </c>
       <c r="W28">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>1.1758511221970355E-2</v>
       </c>
       <c r="X28">
-        <f t="shared" si="21"/>
+        <f t="shared" si="25"/>
         <v>3.7004681240195611E-2</v>
       </c>
       <c r="Y28">
@@ -19467,18 +19467,18 @@
       </c>
       <c r="AD28">
         <f t="shared" si="5"/>
-        <v>90.866868059647501</v>
+        <v>86.053246298476566</v>
       </c>
       <c r="AE28">
         <f t="shared" si="6"/>
-        <v>47.729905925440633</v>
+        <v>53.746933126904295</v>
       </c>
       <c r="AF28">
         <f t="shared" si="7"/>
         <v>20.745686939999999</v>
       </c>
       <c r="AG28">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>48.090310199999998</v>
       </c>
       <c r="AH28">
@@ -19487,7 +19487,7 @@
       </c>
       <c r="AI28">
         <f t="shared" si="9"/>
-        <v>22.716717014911865</v>
+        <v>21.513311574619138</v>
       </c>
       <c r="AJ28">
         <f t="shared" si="10"/>
@@ -19519,6 +19519,6 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Privileged" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>